<commit_message>
update ktp dan kusuka
</commit_message>
<xml_diff>
--- a/analisa_download.xlsx
+++ b/analisa_download.xlsx
@@ -734,11 +734,15 @@
           <t>ASRUL</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -866,11 +870,15 @@
           <t>LA RAKI</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>7403030107780223</v>
-      </c>
-      <c r="G3" t="n">
-        <v>7403030107780223</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>7403030107780223</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>7403030107780223</t>
+        </is>
       </c>
       <c r="H3" t="n">
         <v>82248659536</v>
@@ -998,11 +1006,15 @@
           <t>MUHAMMAD IWAN</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>7403392009870001</v>
-      </c>
-      <c r="G4" t="n">
-        <v>7403392009870001</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>7403392009870001</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>7403392009870001</t>
+        </is>
       </c>
       <c r="H4" t="n">
         <v>82265740892</v>
@@ -1142,11 +1154,15 @@
           <t>MUSRA</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>7403390801800001</v>
-      </c>
-      <c r="G5" t="n">
-        <v>7403390801800001</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>7403390801800001</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>7403390801800001</t>
+        </is>
       </c>
       <c r="H5" t="n">
         <v>81262960963</v>
@@ -1274,11 +1290,15 @@
           <t>RUSLI</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>7403390511860001</v>
-      </c>
-      <c r="G6" t="n">
-        <v>7403390511860001</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>7403390511860001</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>7403390511860001</t>
+        </is>
       </c>
       <c r="H6" t="n">
         <v>84584850398</v>
@@ -1419,11 +1439,15 @@
           <t>RUSLI</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>7403390511860001</v>
-      </c>
-      <c r="G7" t="n">
-        <v>7403390511860001</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>7403390511860001</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>7403390511860001</t>
+        </is>
       </c>
       <c r="H7" t="n">
         <v>84584850398</v>
@@ -1556,11 +1580,15 @@
           <t>DARJO</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>7413080102900001</v>
-      </c>
-      <c r="G8" t="n">
-        <v>7413080102900001</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>7413080102900001</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>7413080102900001</t>
+        </is>
       </c>
       <c r="H8" t="n">
         <v>81245698531</v>
@@ -1700,11 +1728,15 @@
           <t>DARJO</t>
         </is>
       </c>
-      <c r="F9" t="n">
-        <v>7413080102900001</v>
-      </c>
-      <c r="G9" t="n">
-        <v>7413080102900001</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>7413080102900001</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>7413080102900001</t>
+        </is>
       </c>
       <c r="H9" t="n">
         <v>81245698531</v>
@@ -1836,11 +1868,15 @@
           <t>MALAWIN</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>7403020107790204</v>
-      </c>
-      <c r="G10" t="n">
-        <v>7403020107790204</v>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>7403020107790204</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>7403020107790204</t>
+        </is>
       </c>
       <c r="H10" t="n">
         <v>82265879399</v>
@@ -1968,11 +2004,15 @@
           <t>MALAWIN</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>7403020107790204</v>
-      </c>
-      <c r="G11" t="n">
-        <v>7403020107790204</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>7403020107790204</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>7403020107790204</t>
+        </is>
       </c>
       <c r="H11" t="n">
         <v>82265879399</v>
@@ -2100,11 +2140,15 @@
           <t>BAHAR</t>
         </is>
       </c>
-      <c r="F12" t="n">
-        <v>7403050107680212</v>
-      </c>
-      <c r="G12" t="n">
-        <v>7403050107680212</v>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>7403050107680212</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>7403050107680212</t>
+        </is>
       </c>
       <c r="H12" t="n">
         <v>87894760822</v>
@@ -2244,11 +2288,15 @@
           <t>BAHAR</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>7403050107680212</v>
-      </c>
-      <c r="G13" t="n">
-        <v>7403050107680212</v>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>7403050107680212</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>7403050107680212</t>
+        </is>
       </c>
       <c r="H13" t="n">
         <v>87894760822</v>
@@ -2380,11 +2428,15 @@
           <t>FERIS</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>7413060506870001</v>
-      </c>
-      <c r="G14" t="n">
-        <v>7413060506870001</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>7413060506870001</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>7413060506870001</t>
+        </is>
       </c>
       <c r="H14" t="n">
         <v>85747845215</v>
@@ -2512,11 +2564,15 @@
           <t>FERIS</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>7413060506870001</v>
-      </c>
-      <c r="G15" t="n">
-        <v>7413060506870001</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>7413060506870001</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>7413060506870001</t>
+        </is>
       </c>
       <c r="H15" t="n">
         <v>85747845215</v>
@@ -2644,11 +2700,15 @@
           <t>FERIS</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>7413060506870001</v>
-      </c>
-      <c r="G16" t="n">
-        <v>7413060506870001</v>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>7413060506870001</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>7413060506870001</t>
+        </is>
       </c>
       <c r="H16" t="n">
         <v>85747845215</v>
@@ -2776,11 +2836,15 @@
           <t>FERIS</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>7413060506870001</v>
-      </c>
-      <c r="G17" t="n">
-        <v>7413060506870001</v>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>7413060506870001</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>7413060506870001</t>
+        </is>
       </c>
       <c r="H17" t="n">
         <v>85747845215</v>
@@ -2908,11 +2972,15 @@
           <t>ADO</t>
         </is>
       </c>
-      <c r="F18" t="n">
-        <v>7403053112690220</v>
-      </c>
-      <c r="G18" t="n">
-        <v>7403053112690220</v>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>7403053112690220</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>7403053112690220</t>
+        </is>
       </c>
       <c r="H18" t="n">
         <v>85349552536</v>
@@ -3052,11 +3120,15 @@
           <t>ADO</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>7403053112690220</v>
-      </c>
-      <c r="G19" t="n">
-        <v>7403053112690220</v>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>7403053112690220</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>7403053112690220</t>
+        </is>
       </c>
       <c r="H19" t="n">
         <v>85349552536</v>
@@ -3188,11 +3260,15 @@
           <t>SARPIN</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>7403010502850001</v>
-      </c>
-      <c r="G20" t="n">
-        <v>7403010502850001</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>7403010502850001</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>7403010502850001</t>
+        </is>
       </c>
       <c r="H20" t="n">
         <v>82248659536</v>
@@ -3320,11 +3396,15 @@
           <t>MUHAMMAD TAHANG</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>7403020107820212</v>
-      </c>
-      <c r="G21" t="n">
-        <v>7403020107820212</v>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>7403020107820212</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7403020107820212</t>
+        </is>
       </c>
       <c r="H21" t="n">
         <v>82349405893</v>
@@ -3452,11 +3532,15 @@
           <t>hirman</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>7403390107920002</v>
-      </c>
-      <c r="G22" t="n">
-        <v>7403390107920002</v>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>7403390107920002</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>7403390107920002</t>
+        </is>
       </c>
       <c r="H22" t="n">
         <v>84356765208</v>
@@ -3584,11 +3668,15 @@
           <t>ENGGU</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0</v>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H23" t="n">
         <v>82305460879</v>
@@ -3716,11 +3804,15 @@
           <t>ENGGU</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H24" t="n">
         <v>82305460879</v>
@@ -3848,11 +3940,15 @@
           <t>ENGGU</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H25" t="n">
         <v>82305460879</v>
@@ -3980,11 +4076,15 @@
           <t xml:space="preserve">MUH. MARTEN </t>
         </is>
       </c>
-      <c r="F26" t="n">
-        <v>7403361012970001</v>
-      </c>
-      <c r="G26" t="n">
-        <v>7403361012970001</v>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>7403361012970001</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7403361012970001</t>
+        </is>
       </c>
       <c r="H26" t="n">
         <v>82297851797</v>
@@ -4113,11 +4213,15 @@
           <t xml:space="preserve">MUH. MARTEN </t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>7403361012970001</v>
-      </c>
-      <c r="G27" t="n">
-        <v>7403361012970001</v>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>7403361012970001</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>7403361012970001</t>
+        </is>
       </c>
       <c r="H27" t="n">
         <v>82297851797</v>
@@ -4246,11 +4350,15 @@
           <t xml:space="preserve">MUH. MARTEN </t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>7403361012970001</v>
-      </c>
-      <c r="G28" t="n">
-        <v>7403361012970001</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>7403361012970001</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7403361012970001</t>
+        </is>
       </c>
       <c r="H28" t="n">
         <v>82297851797</v>
@@ -4379,11 +4487,15 @@
           <t xml:space="preserve">MUH. MARTEN </t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>7403361012970001</v>
-      </c>
-      <c r="G29" t="n">
-        <v>7403361012970001</v>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>7403361012970001</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>7403361012970001</t>
+        </is>
       </c>
       <c r="H29" t="n">
         <v>82297851797</v>
@@ -4512,11 +4624,15 @@
           <t>SANDI</t>
         </is>
       </c>
-      <c r="F30" t="n">
-        <v>7403051107000202</v>
-      </c>
-      <c r="G30" t="n">
-        <v>7403051107000202</v>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>7403051107000202</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>7403051107000202</t>
+        </is>
       </c>
       <c r="H30" t="n">
         <v>82297541119</v>

</xml_diff>